<commit_message>
chore(fixtures): alinhar modelos de movimentos
</commit_message>
<xml_diff>
--- a/tests/fixtures/modelo_movimentos_operacionais_debito_credito_saldo.xlsx
+++ b/tests/fixtures/modelo_movimentos_operacionais_debito_credito_saldo.xlsx
@@ -19,7 +19,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="3">
+  <fonts count="4">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -34,8 +34,13 @@
     <font>
       <b val="1"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="12"/>
+    </font>
   </fonts>
-  <fills count="4">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
@@ -52,8 +57,18 @@
         <fgColor rgb="00D9EAF7"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF2CC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E2F0D9"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -61,11 +76,25 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="00BFBFBF"/>
+      </left>
+      <right style="thin">
+        <color rgb="00BFBFBF"/>
+      </right>
+      <top style="thin">
+        <color rgb="00BFBFBF"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00BFBFBF"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -73,6 +102,33 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -438,28 +494,28 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M8"/>
+  <dimension ref="A1:M11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
     <col width="18" customWidth="1" min="2" max="2"/>
-    <col width="14" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="14" customWidth="1" min="5" max="5"/>
-    <col width="14" customWidth="1" min="6" max="6"/>
-    <col width="15" customWidth="1" min="7" max="7"/>
-    <col width="16" customWidth="1" min="8" max="8"/>
-    <col width="14" customWidth="1" min="9" max="9"/>
-    <col width="14" customWidth="1" min="10" max="10"/>
-    <col width="17" customWidth="1" min="11" max="11"/>
-    <col width="21" customWidth="1" min="12" max="12"/>
-    <col width="20" customWidth="1" min="13" max="13"/>
+    <col width="38" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="18" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="7" max="7"/>
+    <col width="18" customWidth="1" min="8" max="8"/>
+    <col width="28" customWidth="1" min="9" max="9"/>
+    <col width="20" customWidth="1" min="10" max="10"/>
+    <col width="20" customWidth="1" min="11" max="11"/>
+    <col width="28" customWidth="1" min="12" max="12"/>
+    <col width="28" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Modelo de movimentos operacionais - debito credito e saldo</t>
+    <row r="1" ht="22" customHeight="1">
+      <c r="A1" s="8" t="inlineStr">
+        <is>
+          <t>Modelo de Importacao - Movimentos Operacionais: Debito, Credito e Saldo</t>
         </is>
       </c>
     </row>
@@ -469,6 +525,16 @@
           <t>Empresa</t>
         </is>
       </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>Orientacao</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Preencher razao social ou nome interno</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -476,6 +542,16 @@
           <t>Codigo dominio</t>
         </is>
       </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>Orientacao</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Codigo da empresa no Dominio</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -483,6 +559,16 @@
           <t>CNPJ/CPF</t>
         </is>
       </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>Orientacao</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Obrigatorio</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -490,6 +576,16 @@
           <t>Periodo inicio</t>
         </is>
       </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>Orientacao</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>dd/mm/aaaa</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -497,76 +593,161 @@
           <t>Periodo fim</t>
         </is>
       </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="3" t="inlineStr">
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>Orientacao</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>dd/mm/aaaa</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="22" customHeight="1">
+      <c r="A8" s="9" t="inlineStr">
+        <is>
+          <t>Preencha uma linha por movimento. Colunas amarelas sao obrigatorias; verdes sao opcionais; azuis podem ser preenchidas pelo sistema.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="30" customHeight="1">
+      <c r="A10" s="10" t="inlineStr">
         <is>
           <t>data</t>
         </is>
       </c>
-      <c r="B8" s="3" t="inlineStr">
+      <c r="B10" s="10" t="inlineStr">
         <is>
           <t>conta_financeira</t>
         </is>
       </c>
-      <c r="C8" s="3" t="inlineStr">
+      <c r="C10" s="10" t="inlineStr">
         <is>
           <t>historico</t>
         </is>
       </c>
-      <c r="D8" s="3" t="inlineStr">
+      <c r="D10" s="10" t="inlineStr">
         <is>
           <t>debito</t>
         </is>
       </c>
-      <c r="E8" s="3" t="inlineStr">
+      <c r="E10" s="10" t="inlineStr">
         <is>
           <t>credito</t>
         </is>
       </c>
-      <c r="F8" s="3" t="inlineStr">
+      <c r="F10" s="11" t="inlineStr">
         <is>
           <t>saldo</t>
         </is>
       </c>
-      <c r="G8" s="3" t="inlineStr">
+      <c r="G10" s="11" t="inlineStr">
         <is>
           <t>contrapartida</t>
         </is>
       </c>
-      <c r="H8" s="3" t="inlineStr">
+      <c r="H10" s="11" t="inlineStr">
         <is>
           <t>tipo_movimento</t>
         </is>
       </c>
-      <c r="I8" s="3" t="inlineStr">
+      <c r="I10" s="11" t="inlineStr">
         <is>
           <t>documento</t>
         </is>
       </c>
-      <c r="J8" s="3" t="inlineStr">
+      <c r="J10" s="11" t="inlineStr">
         <is>
           <t>observacao</t>
         </is>
       </c>
-      <c r="K8" s="3" t="inlineStr">
+      <c r="K10" s="12" t="inlineStr">
         <is>
           <t>status_sugerido</t>
         </is>
       </c>
-      <c r="L8" s="3" t="inlineStr">
+      <c r="L10" s="12" t="inlineStr">
         <is>
           <t>confidence_sugerida</t>
         </is>
       </c>
-      <c r="M8" s="3" t="inlineStr">
+      <c r="M10" s="12" t="inlineStr">
         <is>
           <t>mensagem_validacao</t>
         </is>
       </c>
     </row>
+    <row r="11" ht="96" customHeight="1">
+      <c r="A11" s="13" t="inlineStr">
+        <is>
+          <t>Data do movimento. Ex: 31/01/2026</t>
+        </is>
+      </c>
+      <c r="B11" s="13" t="inlineStr">
+        <is>
+          <t>Codigo reduzido da conta financeira/origem. Ex: 10046</t>
+        </is>
+      </c>
+      <c r="C11" s="13" t="inlineStr">
+        <is>
+          <t>Historico original do extrato, planilha ou comprovante.</t>
+        </is>
+      </c>
+      <c r="D11" s="13" t="inlineStr">
+        <is>
+          <t>Valor de saida no extrato. Preencha debito ou credito, nunca ambos.</t>
+        </is>
+      </c>
+      <c r="E11" s="13" t="inlineStr">
+        <is>
+          <t>Valor de entrada no extrato. Preencha credito ou debito, nunca ambos.</t>
+        </is>
+      </c>
+      <c r="F11" s="13" t="inlineStr">
+        <is>
+          <t>Opcional/recomendado. Saldo observado no extrato apos o movimento para conferencia.</t>
+        </is>
+      </c>
+      <c r="G11" s="13" t="inlineStr">
+        <is>
+          <t>Opcional. Codigo reduzido da conta de classificacao/contrapartida, quando conhecido.</t>
+        </is>
+      </c>
+      <c r="H11" s="13" t="inlineStr">
+        <is>
+          <t>Opcional. entrada, saida, transferencia, aplicacao, resgate. Ajuda na validacao.</t>
+        </is>
+      </c>
+      <c r="I11" s="13" t="inlineStr">
+        <is>
+          <t>Opcional. Numero de documento, FITID do OFX, cheque, boleto etc.</t>
+        </is>
+      </c>
+      <c r="J11" s="13" t="inlineStr">
+        <is>
+          <t>Opcional. Comentario livre para revisao.</t>
+        </is>
+      </c>
+      <c r="K11" s="13" t="inlineStr">
+        <is>
+          <t>Preenchido pelo sistema: pendente, sugerido, revisao, aprovado, rejeitado, convertido.</t>
+        </is>
+      </c>
+      <c r="L11" s="13" t="inlineStr">
+        <is>
+          <t>Preenchido pelo sistema: confianca da sugestao.</t>
+        </is>
+      </c>
+      <c r="M11" s="13" t="inlineStr">
+        <is>
+          <t>Preenchido pelo sistema: erros ou alertas de validacao.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="1">
+  <mergeCells count="2">
+    <mergeCell ref="A8:M8"/>
     <mergeCell ref="A1:M1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -579,51 +760,162 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A7"/>
+  <dimension ref="A1:B13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="95" customWidth="1" min="1" max="1"/>
+    <col width="48" customWidth="1" min="1" max="1"/>
+    <col width="48" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="2" t="inlineStr">
+      <c r="A1" s="5" t="inlineStr">
         <is>
           <t>Modelo de movimentos operacionais - debito credito e saldo</t>
         </is>
       </c>
+      <c r="B1" s="5" t="n"/>
+    </row>
+    <row r="2">
+      <c r="A2" s="6" t="inlineStr">
+        <is>
+          <t>Topico</t>
+        </is>
+      </c>
+      <c r="B2" s="6" t="inlineStr">
+        <is>
+          <t>Orientacao</t>
+        </is>
+      </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>Preencha a aba Movimentos sem alterar os nomes das colunas.</t>
+      <c r="A3" s="7" t="inlineStr">
+        <is>
+          <t>Objetivo</t>
+        </is>
+      </c>
+      <c r="B3" s="7" t="inlineStr">
+        <is>
+          <t>Importar movimentos operacionais para classificacao de contrapartida contabil antes da revisao e eventual devolucao da planilha classificada.</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>Use debito para saidas da conta financeira e credito para entradas.</t>
+      <c r="A4" s="7" t="inlineStr">
+        <is>
+          <t>Conta financeira</t>
+        </is>
+      </c>
+      <c r="B4" s="7" t="inlineStr">
+        <is>
+          <t>Use o codigo reduzido da conta financeira ou origem no plano de contas. O sistema valida a conta contra o cadastro da empresa.</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>Preencha exatamente uma entre debito e credito por linha.</t>
+      <c r="A5" s="7" t="inlineStr">
+        <is>
+          <t>Contrapartida</t>
+        </is>
+      </c>
+      <c r="B5" s="7" t="inlineStr">
+        <is>
+          <t>Preencha somente quando souber a conta contabil correta. Deixe em branco quando quiser que o sistema sugira a classificacao.</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>Informe saldo quando quiser permitir conferencia por conta financeira.</t>
+      <c r="A6" s="7" t="inlineStr">
+        <is>
+          <t>Debito e credito</t>
+        </is>
+      </c>
+      <c r="B6" s="7" t="inlineStr">
+        <is>
+          <t>No layout debito, credito e saldo, credito representa entrada na conta financeira e debito representa saida da conta financeira.</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>As colunas status_sugerido, confidence_sugerida e mensagem_validacao sao preenchidas pelo sistema.</t>
+      <c r="A7" s="7" t="inlineStr">
+        <is>
+          <t>Regra por linha</t>
+        </is>
+      </c>
+      <c r="B7" s="7" t="inlineStr">
+        <is>
+          <t>Preencha exatamente uma entre debito e credito por linha. Linha com ambas preenchidas ou ambas vazias deve ser tratada como invalida.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="7" t="inlineStr">
+        <is>
+          <t>Saldo</t>
+        </is>
+      </c>
+      <c r="B8" s="7" t="inlineStr">
+        <is>
+          <t>Informe o saldo observado no extrato quando disponivel. O saldo serve para conferencia por conta financeira e nao entra no aprendizado do classificador.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="7" t="inlineStr">
+        <is>
+          <t>Derivacao contabil</t>
+        </is>
+      </c>
+      <c r="B9" s="7" t="inlineStr">
+        <is>
+          <t>A derivacao debito/credito e calculada a partir da direcao do movimento e da contrapartida informada ou sugerida.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="7" t="inlineStr">
+        <is>
+          <t>Validacao</t>
+        </is>
+      </c>
+      <c r="B10" s="7" t="inlineStr">
+        <is>
+          <t>O sistema valida data, periodo, conta financeira, contrapartida, direcao do valor e coerencia de saldo. Problemas recuperaveis devem gerar aviso por linha ou por lote.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="7" t="inlineStr">
+        <is>
+          <t>Revisao</t>
+        </is>
+      </c>
+      <c r="B11" s="7" t="inlineStr">
+        <is>
+          <t>Linhas sem contrapartida, com baixa confianca ou com alerta devem ser revisadas antes de aprovacao, correcao ou rejeicao.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="7" t="inlineStr">
+        <is>
+          <t>Colunas do sistema</t>
+        </is>
+      </c>
+      <c r="B12" s="7" t="inlineStr">
+        <is>
+          <t>status_sugerido, confidence_sugerida e mensagem_validacao sao preenchidas pelo sistema e devem ficar em branco no preenchimento manual inicial.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="7" t="inlineStr">
+        <is>
+          <t>Dados ficticios</t>
+        </is>
+      </c>
+      <c r="B13" s="7" t="inlineStr">
+        <is>
+          <t>Use exemplos apenas como guia. Nao inclua dados reais de cliente, segredos, documentos sensiveis ou credenciais.</t>
         </is>
       </c>
     </row>
@@ -638,109 +930,293 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G3"/>
+  <dimension ref="A1:K7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="18" customWidth="1" min="1" max="1"/>
-    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="48" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
     <col width="18" customWidth="1" min="3" max="3"/>
-    <col width="18" customWidth="1" min="4" max="4"/>
-    <col width="18" customWidth="1" min="5" max="5"/>
-    <col width="18" customWidth="1" min="6" max="6"/>
-    <col width="18" customWidth="1" min="7" max="7"/>
+    <col width="33" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="15" customWidth="1" min="8" max="8"/>
+    <col width="17" customWidth="1" min="9" max="9"/>
+    <col width="18" customWidth="1" min="10" max="10"/>
+    <col width="43" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="4" t="inlineStr">
-        <is>
-          <t>exemplo</t>
-        </is>
-      </c>
-      <c r="B1" s="4" t="inlineStr">
+      <c r="A1" s="5" t="inlineStr">
+        <is>
+          <t>Exemplos ficticios - Modelo de movimentos operacionais - debito credito e saldo</t>
+        </is>
+      </c>
+      <c r="B1" s="5" t="n"/>
+      <c r="C1" s="5" t="n"/>
+      <c r="D1" s="5" t="n"/>
+      <c r="E1" s="5" t="n"/>
+      <c r="F1" s="5" t="n"/>
+      <c r="G1" s="5" t="n"/>
+      <c r="H1" s="5" t="n"/>
+      <c r="I1" s="5" t="n"/>
+      <c r="J1" s="5" t="n"/>
+      <c r="K1" s="5" t="n"/>
+    </row>
+    <row r="2">
+      <c r="A2" s="6" t="inlineStr">
+        <is>
+          <t>cenario</t>
+        </is>
+      </c>
+      <c r="B2" s="6" t="inlineStr">
         <is>
           <t>data</t>
         </is>
       </c>
-      <c r="C1" s="4" t="inlineStr">
+      <c r="C2" s="6" t="inlineStr">
         <is>
           <t>conta_financeira</t>
         </is>
       </c>
-      <c r="D1" s="4" t="inlineStr">
+      <c r="D2" s="6" t="inlineStr">
         <is>
           <t>historico</t>
         </is>
       </c>
-      <c r="E1" s="4" t="inlineStr">
+      <c r="E2" s="6" t="inlineStr">
         <is>
           <t>debito</t>
         </is>
       </c>
-      <c r="F1" s="4" t="inlineStr">
+      <c r="F2" s="6" t="inlineStr">
         <is>
           <t>credito</t>
         </is>
       </c>
-      <c r="G1" s="4" t="inlineStr">
+      <c r="G2" s="6" t="inlineStr">
         <is>
           <t>saldo</t>
         </is>
       </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>entrada</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>2026-01-05</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>Banco Modelo</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>Recebimento de exemplo</t>
-        </is>
-      </c>
-      <c r="F2" t="n">
+      <c r="H2" s="6" t="inlineStr">
+        <is>
+          <t>contrapartida</t>
+        </is>
+      </c>
+      <c r="I2" s="6" t="inlineStr">
+        <is>
+          <t>debito_derivado</t>
+        </is>
+      </c>
+      <c r="J2" s="6" t="inlineStr">
+        <is>
+          <t>credito_derivado</t>
+        </is>
+      </c>
+      <c r="K2" s="6" t="inlineStr">
+        <is>
+          <t>observacao</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="7" t="inlineStr">
+        <is>
+          <t>Recebimento</t>
+        </is>
+      </c>
+      <c r="B3" s="7" t="inlineStr">
+        <is>
+          <t>05/01/2026</t>
+        </is>
+      </c>
+      <c r="C3" s="7" t="n">
+        <v>10046</v>
+      </c>
+      <c r="D3" s="7" t="inlineStr">
+        <is>
+          <t>RECEBIMENTO CLIENTE FICTICIO</t>
+        </is>
+      </c>
+      <c r="E3" s="7" t="n"/>
+      <c r="F3" s="7" t="n">
         <v>1500</v>
       </c>
-      <c r="G2" t="n">
+      <c r="G3" s="7" t="n">
         <v>2500</v>
       </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>saida</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>2026-01-06</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>Banco Modelo</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>Pagamento de exemplo</t>
-        </is>
-      </c>
-      <c r="E3" t="n">
+      <c r="H3" s="7" t="n">
+        <v>10722</v>
+      </c>
+      <c r="I3" s="7" t="n">
+        <v>10046</v>
+      </c>
+      <c r="J3" s="7" t="n">
+        <v>10722</v>
+      </c>
+      <c r="K3" s="7" t="inlineStr">
+        <is>
+          <t>Credito do extrato aumenta banco.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="7" t="inlineStr">
+        <is>
+          <t>Pagamento</t>
+        </is>
+      </c>
+      <c r="B4" s="7" t="inlineStr">
+        <is>
+          <t>06/01/2026</t>
+        </is>
+      </c>
+      <c r="C4" s="7" t="n">
+        <v>10046</v>
+      </c>
+      <c r="D4" s="7" t="inlineStr">
+        <is>
+          <t>PAGAMENTO FORNECEDOR FICTICIO</t>
+        </is>
+      </c>
+      <c r="E4" s="7" t="n">
         <v>300</v>
       </c>
-      <c r="G3" t="n">
+      <c r="F4" s="7" t="n"/>
+      <c r="G4" s="7" t="n">
         <v>2200</v>
+      </c>
+      <c r="H4" s="7" t="n">
+        <v>103382</v>
+      </c>
+      <c r="I4" s="7" t="n">
+        <v>103382</v>
+      </c>
+      <c r="J4" s="7" t="n">
+        <v>10046</v>
+      </c>
+      <c r="K4" s="7" t="inlineStr">
+        <is>
+          <t>Debito do extrato reduz banco.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="7" t="inlineStr">
+        <is>
+          <t>Aplicacao</t>
+        </is>
+      </c>
+      <c r="B5" s="7" t="inlineStr">
+        <is>
+          <t>07/01/2026</t>
+        </is>
+      </c>
+      <c r="C5" s="7" t="n">
+        <v>10046</v>
+      </c>
+      <c r="D5" s="7" t="inlineStr">
+        <is>
+          <t>APLICACAO FINANCEIRA FICTICIA</t>
+        </is>
+      </c>
+      <c r="E5" s="7" t="n">
+        <v>600</v>
+      </c>
+      <c r="F5" s="7" t="n"/>
+      <c r="G5" s="7" t="n">
+        <v>1600</v>
+      </c>
+      <c r="H5" s="7" t="n">
+        <v>10126</v>
+      </c>
+      <c r="I5" s="7" t="n">
+        <v>10126</v>
+      </c>
+      <c r="J5" s="7" t="n">
+        <v>10046</v>
+      </c>
+      <c r="K5" s="7" t="inlineStr">
+        <is>
+          <t>Saida do banco para aplicacao.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="7" t="inlineStr">
+        <is>
+          <t>Resgate</t>
+        </is>
+      </c>
+      <c r="B6" s="7" t="inlineStr">
+        <is>
+          <t>08/01/2026</t>
+        </is>
+      </c>
+      <c r="C6" s="7" t="n">
+        <v>10046</v>
+      </c>
+      <c r="D6" s="7" t="inlineStr">
+        <is>
+          <t>RESGATE APLICACAO FICTICIA</t>
+        </is>
+      </c>
+      <c r="E6" s="7" t="n"/>
+      <c r="F6" s="7" t="n">
+        <v>400</v>
+      </c>
+      <c r="G6" s="7" t="n">
+        <v>2000</v>
+      </c>
+      <c r="H6" s="7" t="n">
+        <v>10126</v>
+      </c>
+      <c r="I6" s="7" t="n">
+        <v>10046</v>
+      </c>
+      <c r="J6" s="7" t="n">
+        <v>10126</v>
+      </c>
+      <c r="K6" s="7" t="inlineStr">
+        <is>
+          <t>Entrada no banco por resgate.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="7" t="inlineStr">
+        <is>
+          <t>Classificar</t>
+        </is>
+      </c>
+      <c r="B7" s="7" t="inlineStr">
+        <is>
+          <t>09/01/2026</t>
+        </is>
+      </c>
+      <c r="C7" s="7" t="n">
+        <v>10046</v>
+      </c>
+      <c r="D7" s="7" t="inlineStr">
+        <is>
+          <t>PAGAMENTO SERVICO A CLASSIFICAR</t>
+        </is>
+      </c>
+      <c r="E7" s="7" t="n">
+        <v>250</v>
+      </c>
+      <c r="F7" s="7" t="n"/>
+      <c r="G7" s="7" t="n">
+        <v>1750</v>
+      </c>
+      <c r="H7" s="7" t="n"/>
+      <c r="I7" s="7" t="n"/>
+      <c r="J7" s="7" t="n"/>
+      <c r="K7" s="7" t="inlineStr">
+        <is>
+          <t>Sem contrapartida para o sistema sugerir.</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore(fixtures): alinhar modelos de movimentos (#464)
* chore(fixtures): alinhar modelos de movimentos

* Merge branch 'main' into chore/fixtures-instrucoes-movimentos
</commit_message>
<xml_diff>
--- a/tests/fixtures/modelo_movimentos_operacionais_debito_credito_saldo.xlsx
+++ b/tests/fixtures/modelo_movimentos_operacionais_debito_credito_saldo.xlsx
@@ -19,7 +19,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="3">
+  <fonts count="4">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -34,8 +34,13 @@
     <font>
       <b val="1"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="12"/>
+    </font>
   </fonts>
-  <fills count="4">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
@@ -52,8 +57,18 @@
         <fgColor rgb="00D9EAF7"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF2CC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E2F0D9"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -61,11 +76,25 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="00BFBFBF"/>
+      </left>
+      <right style="thin">
+        <color rgb="00BFBFBF"/>
+      </right>
+      <top style="thin">
+        <color rgb="00BFBFBF"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00BFBFBF"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -73,6 +102,33 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -438,28 +494,28 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M8"/>
+  <dimension ref="A1:M11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
     <col width="18" customWidth="1" min="2" max="2"/>
-    <col width="14" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="14" customWidth="1" min="5" max="5"/>
-    <col width="14" customWidth="1" min="6" max="6"/>
-    <col width="15" customWidth="1" min="7" max="7"/>
-    <col width="16" customWidth="1" min="8" max="8"/>
-    <col width="14" customWidth="1" min="9" max="9"/>
-    <col width="14" customWidth="1" min="10" max="10"/>
-    <col width="17" customWidth="1" min="11" max="11"/>
-    <col width="21" customWidth="1" min="12" max="12"/>
-    <col width="20" customWidth="1" min="13" max="13"/>
+    <col width="38" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="18" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="7" max="7"/>
+    <col width="18" customWidth="1" min="8" max="8"/>
+    <col width="28" customWidth="1" min="9" max="9"/>
+    <col width="20" customWidth="1" min="10" max="10"/>
+    <col width="20" customWidth="1" min="11" max="11"/>
+    <col width="28" customWidth="1" min="12" max="12"/>
+    <col width="28" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Modelo de movimentos operacionais - debito credito e saldo</t>
+    <row r="1" ht="22" customHeight="1">
+      <c r="A1" s="8" t="inlineStr">
+        <is>
+          <t>Modelo de Importacao - Movimentos Operacionais: Debito, Credito e Saldo</t>
         </is>
       </c>
     </row>
@@ -469,6 +525,16 @@
           <t>Empresa</t>
         </is>
       </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>Orientacao</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Preencher razao social ou nome interno</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -476,6 +542,16 @@
           <t>Codigo dominio</t>
         </is>
       </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>Orientacao</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Codigo da empresa no Dominio</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -483,6 +559,16 @@
           <t>CNPJ/CPF</t>
         </is>
       </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>Orientacao</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Obrigatorio</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -490,6 +576,16 @@
           <t>Periodo inicio</t>
         </is>
       </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>Orientacao</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>dd/mm/aaaa</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -497,76 +593,161 @@
           <t>Periodo fim</t>
         </is>
       </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="3" t="inlineStr">
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>Orientacao</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>dd/mm/aaaa</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="22" customHeight="1">
+      <c r="A8" s="9" t="inlineStr">
+        <is>
+          <t>Preencha uma linha por movimento. Colunas amarelas sao obrigatorias; verdes sao opcionais; azuis podem ser preenchidas pelo sistema.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="30" customHeight="1">
+      <c r="A10" s="10" t="inlineStr">
         <is>
           <t>data</t>
         </is>
       </c>
-      <c r="B8" s="3" t="inlineStr">
+      <c r="B10" s="10" t="inlineStr">
         <is>
           <t>conta_financeira</t>
         </is>
       </c>
-      <c r="C8" s="3" t="inlineStr">
+      <c r="C10" s="10" t="inlineStr">
         <is>
           <t>historico</t>
         </is>
       </c>
-      <c r="D8" s="3" t="inlineStr">
+      <c r="D10" s="10" t="inlineStr">
         <is>
           <t>debito</t>
         </is>
       </c>
-      <c r="E8" s="3" t="inlineStr">
+      <c r="E10" s="10" t="inlineStr">
         <is>
           <t>credito</t>
         </is>
       </c>
-      <c r="F8" s="3" t="inlineStr">
+      <c r="F10" s="11" t="inlineStr">
         <is>
           <t>saldo</t>
         </is>
       </c>
-      <c r="G8" s="3" t="inlineStr">
+      <c r="G10" s="11" t="inlineStr">
         <is>
           <t>contrapartida</t>
         </is>
       </c>
-      <c r="H8" s="3" t="inlineStr">
+      <c r="H10" s="11" t="inlineStr">
         <is>
           <t>tipo_movimento</t>
         </is>
       </c>
-      <c r="I8" s="3" t="inlineStr">
+      <c r="I10" s="11" t="inlineStr">
         <is>
           <t>documento</t>
         </is>
       </c>
-      <c r="J8" s="3" t="inlineStr">
+      <c r="J10" s="11" t="inlineStr">
         <is>
           <t>observacao</t>
         </is>
       </c>
-      <c r="K8" s="3" t="inlineStr">
+      <c r="K10" s="12" t="inlineStr">
         <is>
           <t>status_sugerido</t>
         </is>
       </c>
-      <c r="L8" s="3" t="inlineStr">
+      <c r="L10" s="12" t="inlineStr">
         <is>
           <t>confidence_sugerida</t>
         </is>
       </c>
-      <c r="M8" s="3" t="inlineStr">
+      <c r="M10" s="12" t="inlineStr">
         <is>
           <t>mensagem_validacao</t>
         </is>
       </c>
     </row>
+    <row r="11" ht="96" customHeight="1">
+      <c r="A11" s="13" t="inlineStr">
+        <is>
+          <t>Data do movimento. Ex: 31/01/2026</t>
+        </is>
+      </c>
+      <c r="B11" s="13" t="inlineStr">
+        <is>
+          <t>Codigo reduzido da conta financeira/origem. Ex: 10046</t>
+        </is>
+      </c>
+      <c r="C11" s="13" t="inlineStr">
+        <is>
+          <t>Historico original do extrato, planilha ou comprovante.</t>
+        </is>
+      </c>
+      <c r="D11" s="13" t="inlineStr">
+        <is>
+          <t>Valor de saida no extrato. Preencha debito ou credito, nunca ambos.</t>
+        </is>
+      </c>
+      <c r="E11" s="13" t="inlineStr">
+        <is>
+          <t>Valor de entrada no extrato. Preencha credito ou debito, nunca ambos.</t>
+        </is>
+      </c>
+      <c r="F11" s="13" t="inlineStr">
+        <is>
+          <t>Opcional/recomendado. Saldo observado no extrato apos o movimento para conferencia.</t>
+        </is>
+      </c>
+      <c r="G11" s="13" t="inlineStr">
+        <is>
+          <t>Opcional. Codigo reduzido da conta de classificacao/contrapartida, quando conhecido.</t>
+        </is>
+      </c>
+      <c r="H11" s="13" t="inlineStr">
+        <is>
+          <t>Opcional. entrada, saida, transferencia, aplicacao, resgate. Ajuda na validacao.</t>
+        </is>
+      </c>
+      <c r="I11" s="13" t="inlineStr">
+        <is>
+          <t>Opcional. Numero de documento, FITID do OFX, cheque, boleto etc.</t>
+        </is>
+      </c>
+      <c r="J11" s="13" t="inlineStr">
+        <is>
+          <t>Opcional. Comentario livre para revisao.</t>
+        </is>
+      </c>
+      <c r="K11" s="13" t="inlineStr">
+        <is>
+          <t>Preenchido pelo sistema: pendente, sugerido, revisao, aprovado, rejeitado, convertido.</t>
+        </is>
+      </c>
+      <c r="L11" s="13" t="inlineStr">
+        <is>
+          <t>Preenchido pelo sistema: confianca da sugestao.</t>
+        </is>
+      </c>
+      <c r="M11" s="13" t="inlineStr">
+        <is>
+          <t>Preenchido pelo sistema: erros ou alertas de validacao.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="1">
+  <mergeCells count="2">
+    <mergeCell ref="A8:M8"/>
     <mergeCell ref="A1:M1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -579,51 +760,162 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A7"/>
+  <dimension ref="A1:B13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="95" customWidth="1" min="1" max="1"/>
+    <col width="48" customWidth="1" min="1" max="1"/>
+    <col width="48" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="2" t="inlineStr">
+      <c r="A1" s="5" t="inlineStr">
         <is>
           <t>Modelo de movimentos operacionais - debito credito e saldo</t>
         </is>
       </c>
+      <c r="B1" s="5" t="n"/>
+    </row>
+    <row r="2">
+      <c r="A2" s="6" t="inlineStr">
+        <is>
+          <t>Topico</t>
+        </is>
+      </c>
+      <c r="B2" s="6" t="inlineStr">
+        <is>
+          <t>Orientacao</t>
+        </is>
+      </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>Preencha a aba Movimentos sem alterar os nomes das colunas.</t>
+      <c r="A3" s="7" t="inlineStr">
+        <is>
+          <t>Objetivo</t>
+        </is>
+      </c>
+      <c r="B3" s="7" t="inlineStr">
+        <is>
+          <t>Importar movimentos operacionais para classificacao de contrapartida contabil antes da revisao e eventual devolucao da planilha classificada.</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>Use debito para saidas da conta financeira e credito para entradas.</t>
+      <c r="A4" s="7" t="inlineStr">
+        <is>
+          <t>Conta financeira</t>
+        </is>
+      </c>
+      <c r="B4" s="7" t="inlineStr">
+        <is>
+          <t>Use o codigo reduzido da conta financeira ou origem no plano de contas. O sistema valida a conta contra o cadastro da empresa.</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>Preencha exatamente uma entre debito e credito por linha.</t>
+      <c r="A5" s="7" t="inlineStr">
+        <is>
+          <t>Contrapartida</t>
+        </is>
+      </c>
+      <c r="B5" s="7" t="inlineStr">
+        <is>
+          <t>Preencha somente quando souber a conta contabil correta. Deixe em branco quando quiser que o sistema sugira a classificacao.</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>Informe saldo quando quiser permitir conferencia por conta financeira.</t>
+      <c r="A6" s="7" t="inlineStr">
+        <is>
+          <t>Debito e credito</t>
+        </is>
+      </c>
+      <c r="B6" s="7" t="inlineStr">
+        <is>
+          <t>No layout debito, credito e saldo, credito representa entrada na conta financeira e debito representa saida da conta financeira.</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>As colunas status_sugerido, confidence_sugerida e mensagem_validacao sao preenchidas pelo sistema.</t>
+      <c r="A7" s="7" t="inlineStr">
+        <is>
+          <t>Regra por linha</t>
+        </is>
+      </c>
+      <c r="B7" s="7" t="inlineStr">
+        <is>
+          <t>Preencha exatamente uma entre debito e credito por linha. Linha com ambas preenchidas ou ambas vazias deve ser tratada como invalida.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="7" t="inlineStr">
+        <is>
+          <t>Saldo</t>
+        </is>
+      </c>
+      <c r="B8" s="7" t="inlineStr">
+        <is>
+          <t>Informe o saldo observado no extrato quando disponivel. O saldo serve para conferencia por conta financeira e nao entra no aprendizado do classificador.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="7" t="inlineStr">
+        <is>
+          <t>Derivacao contabil</t>
+        </is>
+      </c>
+      <c r="B9" s="7" t="inlineStr">
+        <is>
+          <t>A derivacao debito/credito e calculada a partir da direcao do movimento e da contrapartida informada ou sugerida.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="7" t="inlineStr">
+        <is>
+          <t>Validacao</t>
+        </is>
+      </c>
+      <c r="B10" s="7" t="inlineStr">
+        <is>
+          <t>O sistema valida data, periodo, conta financeira, contrapartida, direcao do valor e coerencia de saldo. Problemas recuperaveis devem gerar aviso por linha ou por lote.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="7" t="inlineStr">
+        <is>
+          <t>Revisao</t>
+        </is>
+      </c>
+      <c r="B11" s="7" t="inlineStr">
+        <is>
+          <t>Linhas sem contrapartida, com baixa confianca ou com alerta devem ser revisadas antes de aprovacao, correcao ou rejeicao.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="7" t="inlineStr">
+        <is>
+          <t>Colunas do sistema</t>
+        </is>
+      </c>
+      <c r="B12" s="7" t="inlineStr">
+        <is>
+          <t>status_sugerido, confidence_sugerida e mensagem_validacao sao preenchidas pelo sistema e devem ficar em branco no preenchimento manual inicial.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="7" t="inlineStr">
+        <is>
+          <t>Dados ficticios</t>
+        </is>
+      </c>
+      <c r="B13" s="7" t="inlineStr">
+        <is>
+          <t>Use exemplos apenas como guia. Nao inclua dados reais de cliente, segredos, documentos sensiveis ou credenciais.</t>
         </is>
       </c>
     </row>
@@ -638,109 +930,293 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G3"/>
+  <dimension ref="A1:K7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="18" customWidth="1" min="1" max="1"/>
-    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="48" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
     <col width="18" customWidth="1" min="3" max="3"/>
-    <col width="18" customWidth="1" min="4" max="4"/>
-    <col width="18" customWidth="1" min="5" max="5"/>
-    <col width="18" customWidth="1" min="6" max="6"/>
-    <col width="18" customWidth="1" min="7" max="7"/>
+    <col width="33" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="15" customWidth="1" min="8" max="8"/>
+    <col width="17" customWidth="1" min="9" max="9"/>
+    <col width="18" customWidth="1" min="10" max="10"/>
+    <col width="43" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="4" t="inlineStr">
-        <is>
-          <t>exemplo</t>
-        </is>
-      </c>
-      <c r="B1" s="4" t="inlineStr">
+      <c r="A1" s="5" t="inlineStr">
+        <is>
+          <t>Exemplos ficticios - Modelo de movimentos operacionais - debito credito e saldo</t>
+        </is>
+      </c>
+      <c r="B1" s="5" t="n"/>
+      <c r="C1" s="5" t="n"/>
+      <c r="D1" s="5" t="n"/>
+      <c r="E1" s="5" t="n"/>
+      <c r="F1" s="5" t="n"/>
+      <c r="G1" s="5" t="n"/>
+      <c r="H1" s="5" t="n"/>
+      <c r="I1" s="5" t="n"/>
+      <c r="J1" s="5" t="n"/>
+      <c r="K1" s="5" t="n"/>
+    </row>
+    <row r="2">
+      <c r="A2" s="6" t="inlineStr">
+        <is>
+          <t>cenario</t>
+        </is>
+      </c>
+      <c r="B2" s="6" t="inlineStr">
         <is>
           <t>data</t>
         </is>
       </c>
-      <c r="C1" s="4" t="inlineStr">
+      <c r="C2" s="6" t="inlineStr">
         <is>
           <t>conta_financeira</t>
         </is>
       </c>
-      <c r="D1" s="4" t="inlineStr">
+      <c r="D2" s="6" t="inlineStr">
         <is>
           <t>historico</t>
         </is>
       </c>
-      <c r="E1" s="4" t="inlineStr">
+      <c r="E2" s="6" t="inlineStr">
         <is>
           <t>debito</t>
         </is>
       </c>
-      <c r="F1" s="4" t="inlineStr">
+      <c r="F2" s="6" t="inlineStr">
         <is>
           <t>credito</t>
         </is>
       </c>
-      <c r="G1" s="4" t="inlineStr">
+      <c r="G2" s="6" t="inlineStr">
         <is>
           <t>saldo</t>
         </is>
       </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>entrada</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>2026-01-05</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>Banco Modelo</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>Recebimento de exemplo</t>
-        </is>
-      </c>
-      <c r="F2" t="n">
+      <c r="H2" s="6" t="inlineStr">
+        <is>
+          <t>contrapartida</t>
+        </is>
+      </c>
+      <c r="I2" s="6" t="inlineStr">
+        <is>
+          <t>debito_derivado</t>
+        </is>
+      </c>
+      <c r="J2" s="6" t="inlineStr">
+        <is>
+          <t>credito_derivado</t>
+        </is>
+      </c>
+      <c r="K2" s="6" t="inlineStr">
+        <is>
+          <t>observacao</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="7" t="inlineStr">
+        <is>
+          <t>Recebimento</t>
+        </is>
+      </c>
+      <c r="B3" s="7" t="inlineStr">
+        <is>
+          <t>05/01/2026</t>
+        </is>
+      </c>
+      <c r="C3" s="7" t="n">
+        <v>10046</v>
+      </c>
+      <c r="D3" s="7" t="inlineStr">
+        <is>
+          <t>RECEBIMENTO CLIENTE FICTICIO</t>
+        </is>
+      </c>
+      <c r="E3" s="7" t="n"/>
+      <c r="F3" s="7" t="n">
         <v>1500</v>
       </c>
-      <c r="G2" t="n">
+      <c r="G3" s="7" t="n">
         <v>2500</v>
       </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>saida</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>2026-01-06</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>Banco Modelo</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>Pagamento de exemplo</t>
-        </is>
-      </c>
-      <c r="E3" t="n">
+      <c r="H3" s="7" t="n">
+        <v>10722</v>
+      </c>
+      <c r="I3" s="7" t="n">
+        <v>10046</v>
+      </c>
+      <c r="J3" s="7" t="n">
+        <v>10722</v>
+      </c>
+      <c r="K3" s="7" t="inlineStr">
+        <is>
+          <t>Credito do extrato aumenta banco.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="7" t="inlineStr">
+        <is>
+          <t>Pagamento</t>
+        </is>
+      </c>
+      <c r="B4" s="7" t="inlineStr">
+        <is>
+          <t>06/01/2026</t>
+        </is>
+      </c>
+      <c r="C4" s="7" t="n">
+        <v>10046</v>
+      </c>
+      <c r="D4" s="7" t="inlineStr">
+        <is>
+          <t>PAGAMENTO FORNECEDOR FICTICIO</t>
+        </is>
+      </c>
+      <c r="E4" s="7" t="n">
         <v>300</v>
       </c>
-      <c r="G3" t="n">
+      <c r="F4" s="7" t="n"/>
+      <c r="G4" s="7" t="n">
         <v>2200</v>
+      </c>
+      <c r="H4" s="7" t="n">
+        <v>103382</v>
+      </c>
+      <c r="I4" s="7" t="n">
+        <v>103382</v>
+      </c>
+      <c r="J4" s="7" t="n">
+        <v>10046</v>
+      </c>
+      <c r="K4" s="7" t="inlineStr">
+        <is>
+          <t>Debito do extrato reduz banco.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="7" t="inlineStr">
+        <is>
+          <t>Aplicacao</t>
+        </is>
+      </c>
+      <c r="B5" s="7" t="inlineStr">
+        <is>
+          <t>07/01/2026</t>
+        </is>
+      </c>
+      <c r="C5" s="7" t="n">
+        <v>10046</v>
+      </c>
+      <c r="D5" s="7" t="inlineStr">
+        <is>
+          <t>APLICACAO FINANCEIRA FICTICIA</t>
+        </is>
+      </c>
+      <c r="E5" s="7" t="n">
+        <v>600</v>
+      </c>
+      <c r="F5" s="7" t="n"/>
+      <c r="G5" s="7" t="n">
+        <v>1600</v>
+      </c>
+      <c r="H5" s="7" t="n">
+        <v>10126</v>
+      </c>
+      <c r="I5" s="7" t="n">
+        <v>10126</v>
+      </c>
+      <c r="J5" s="7" t="n">
+        <v>10046</v>
+      </c>
+      <c r="K5" s="7" t="inlineStr">
+        <is>
+          <t>Saida do banco para aplicacao.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="7" t="inlineStr">
+        <is>
+          <t>Resgate</t>
+        </is>
+      </c>
+      <c r="B6" s="7" t="inlineStr">
+        <is>
+          <t>08/01/2026</t>
+        </is>
+      </c>
+      <c r="C6" s="7" t="n">
+        <v>10046</v>
+      </c>
+      <c r="D6" s="7" t="inlineStr">
+        <is>
+          <t>RESGATE APLICACAO FICTICIA</t>
+        </is>
+      </c>
+      <c r="E6" s="7" t="n"/>
+      <c r="F6" s="7" t="n">
+        <v>400</v>
+      </c>
+      <c r="G6" s="7" t="n">
+        <v>2000</v>
+      </c>
+      <c r="H6" s="7" t="n">
+        <v>10126</v>
+      </c>
+      <c r="I6" s="7" t="n">
+        <v>10046</v>
+      </c>
+      <c r="J6" s="7" t="n">
+        <v>10126</v>
+      </c>
+      <c r="K6" s="7" t="inlineStr">
+        <is>
+          <t>Entrada no banco por resgate.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="7" t="inlineStr">
+        <is>
+          <t>Classificar</t>
+        </is>
+      </c>
+      <c r="B7" s="7" t="inlineStr">
+        <is>
+          <t>09/01/2026</t>
+        </is>
+      </c>
+      <c r="C7" s="7" t="n">
+        <v>10046</v>
+      </c>
+      <c r="D7" s="7" t="inlineStr">
+        <is>
+          <t>PAGAMENTO SERVICO A CLASSIFICAR</t>
+        </is>
+      </c>
+      <c r="E7" s="7" t="n">
+        <v>250</v>
+      </c>
+      <c r="F7" s="7" t="n"/>
+      <c r="G7" s="7" t="n">
+        <v>1750</v>
+      </c>
+      <c r="H7" s="7" t="n"/>
+      <c r="I7" s="7" t="n"/>
+      <c r="J7" s="7" t="n"/>
+      <c r="K7" s="7" t="inlineStr">
+        <is>
+          <t>Sem contrapartida para o sistema sugerir.</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>